<commit_message>
Optimize 3D rendering performance and add planet-to-ring connectivity
Cache instanced meshes and typed arrays to avoid per-frame allocations,
pre-compute color objects for link rendering, add FPS counter, use O(1)
Map/Set lookups in network graph building and max-flow BFS, add bucketed
Gbps cache, and connect planets directly to their nearest ring satellites.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/marslink_analysis.xlsx
+++ b/analysis/marslink_analysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fits" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fits" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7429,7 +7429,7 @@
         <v>0.07345462979050342</v>
       </c>
       <c r="C3" t="n">
-        <v>0.007717406724392821</v>
+        <v>0.007717406724367332</v>
       </c>
     </row>
     <row r="4">

</xml_diff>